<commit_message>
Highlight unpublished in HIL Mux Layout Published column too
Apply the same amber + bold emphasis to the "no" Published cells in
the HIL Mux Layout linear export table, matching the Component Matrix.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hil_i2c_components.xlsx
+++ b/hil_i2c_components.xlsx
@@ -16781,7 +16781,7 @@
         </is>
       </c>
       <c r="BY30" s="28" t="inlineStr"/>
-      <c r="BZ30" s="28" t="inlineStr">
+      <c r="BZ30" s="9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -17383,7 +17383,7 @@
         </is>
       </c>
       <c r="BY34" s="28" t="inlineStr"/>
-      <c r="BZ34" s="28" t="inlineStr">
+      <c r="BZ34" s="9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -22465,7 +22465,7 @@
         </is>
       </c>
       <c r="BY105" s="31" t="inlineStr"/>
-      <c r="BZ105" s="31" t="inlineStr">
+      <c r="BZ105" s="9" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>